<commit_message>
Add company and decision-maker emails to the lead list
Company emails are those published on each company's own site
(imprint/contact pages); decision-maker emails come from Apify's
LinkedIn profile email search (with status/score) or the company site.
No addresses are guessed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7WGfj2Ei9TMEtkpj84W2s
</commit_message>
<xml_diff>
--- a/reports/callypso_engage_europe_turkish_ecommerce_leads.xlsx
+++ b/reports/callypso_engage_europe_turkish_ecommerce_leads.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$W$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$AC$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W82"/>
+  <dimension ref="A1:AC82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -453,6 +453,12 @@
     <col width="62" customWidth="1" min="21" max="21"/>
     <col width="18" customWidth="1" min="22" max="22"/>
     <col width="62" customWidth="1" min="23" max="23"/>
+    <col width="52" customWidth="1" min="24" max="24"/>
+    <col width="46" customWidth="1" min="25" max="25"/>
+    <col width="32" customWidth="1" min="26" max="26"/>
+    <col width="61" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,6 +577,36 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Company Email</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Company Email Source URL</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Email</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Email Source</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary Email</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary Email Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -688,6 +724,20 @@
           <t>LinkedIn page matched by name (manually confirmed: same company, no/related website)</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>ecommerce@aytac.co.uk, customerservice@aytac.co.uk</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>https://aytacfood.co.uk</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -793,6 +843,28 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>help@limanonline.com</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>https://www.limanonline.com</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>talip.altintas@limanonline.com</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Apify LinkedIn email search: risky (score 60)</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -898,6 +970,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>hello@bodrumfoods.co.uk</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>https://www.bodrumfoods.co.uk</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1003,6 +1089,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>help@bonvila.com, hello@bonvila.com</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>https://bonvila.com</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1092,6 +1192,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>info@edensmarket.be</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>https://edensmarket.be/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1181,6 +1295,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>contact@istanbul-market.com</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>https://www.istanbul-market.com</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1278,6 +1406,28 @@
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>emin.meteriz@cici-home.com, kontakt@cici-home.de</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>https://cici-home.com/impressum</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>emin.meteriz@cici-home.com</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Published on company site (https://cici-home.com/impressum)</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1367,6 +1517,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>shop@foodpaket.de</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>https://www.foodpaket.de/pages/impressum</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1452,6 +1616,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>admin@turkmarketi.de</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>https://www.turkmarketi.de</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1557,6 +1735,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>orders.ela@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>https://elawonen.nl</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1642,6 +1834,20 @@
           <t>Outside priority countries; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>info@evim.ch</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>https://evim.ch</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1759,6 +1965,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>online@anthap.co.uk, info@anthap.co.uk</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>https://www.anthap.co.uk</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1852,6 +2072,12 @@
           <t>LinkedIn page matched by name (manually confirmed: same company, no/related website); No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1945,6 +2171,12 @@
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2030,6 +2262,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2123,6 +2361,12 @@
           <t>LinkedIn page matched by name (manually confirmed: same company, no/related website); No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2220,6 +2464,20 @@
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>info@bakkal.eu</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>https://www.bakkal.eu/policies/legal-notice</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2305,6 +2563,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2390,6 +2654,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2475,6 +2745,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2560,6 +2836,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2657,6 +2939,20 @@
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>marketing@hatay.de, shop@hatay.de</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>https://hatay.de</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2762,6 +3058,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>support@kochdichtuerkisch.de</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>https://shop.kochdichturkisch.de</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2851,6 +3161,20 @@
           <t>Karaca.nl appears to be run by same ecosystem - not merged; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>info@gulcanhome.eu</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>https://gulcanhome.eu</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2936,6 +3260,20 @@
           <t>Outside priority countries; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>kontakt@bizimkiler.ch</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>https://bizimkiler.ch</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3021,6 +3359,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>info@goturkishfood.com</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>https://goturkishfood.com</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3122,6 +3474,20 @@
           <t>LinkedIn page matched by name (manually confirmed: same company, no/related website)</t>
         </is>
       </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>turksarayi@hotmail.com</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>https://turksarayi.com/pages/contact-us</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3207,6 +3573,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3292,6 +3664,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3381,6 +3759,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>info@hepsikapinda-shop.com</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>https://hepsikapinda-shop.com</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3470,6 +3862,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>info@capadocia.de</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>https://capadocia.de</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3563,6 +3969,20 @@
           <t>LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>info@hepsi-markt.de</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>https://hepsi-markt.de/impressum</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3656,6 +4076,20 @@
           <t>LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>kundenservice@morgenmarkt.de</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>https://morgenmarkt.de</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3745,6 +4179,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>info@tazecik.de</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>https://www.tazecik.de/pages/impressum</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3838,6 +4286,20 @@
           <t>Grocery: high repeat; LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>info@bakal.de</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>https://bakal.de/impressum</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3927,6 +4389,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>info@ekselansonline.com</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>https://ekselansonline.com</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4016,6 +4492,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>info@turkuazmarket.nl</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>https://turkuazmarket.nl/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4101,6 +4591,12 @@
           <t>Outside priority countries; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4202,6 +4698,20 @@
           <t>LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>info@zmcexport.com</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>https://mughegourmet.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4291,6 +4801,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>office@beslershop.de</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>https://beslermarkt.de</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4400,6 +4924,20 @@
         </is>
       </c>
       <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>shop@evimhome.de</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>https://evimhome.de/pages/impressum</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4489,6 +5027,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>shop@ulusoy-export.de</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>https://ulusoy-export.de/impressum</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4574,6 +5126,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4663,6 +5221,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>info@karakushome.com</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>https://karakushome.com</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4756,6 +5328,20 @@
           <t>LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>info@olijfoliemarkt.nl</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>https://olijfoliemarkt.nl</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4841,6 +5427,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>orders@bestgrocery.co.uk</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>https://bestgrocery.co.uk</t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4926,6 +5526,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>merhababoutique786@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>https://merhababoutique.com</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5015,6 +5629,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>office@bellaneva.com</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>https://bellaneva.com</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5104,6 +5732,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>info@alyadress.de</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>https://alyadress.de/policies/legal-notice</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5193,6 +5835,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>info@back-lava.de, grandcafe@back-lava.de</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>https://back-lava.de</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5282,6 +5938,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>info@naturdeluxe.com</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>https://www.naturdeluxe.com</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5367,6 +6037,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5452,6 +6128,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>info@anamarket.nl</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>https://anamarket.nl</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5549,6 +6239,28 @@
         </is>
       </c>
       <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>info@yasamfood.com</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>https://yasamfood.com</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>d.ercel@yasamfood.com</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>Apify LinkedIn email search: valid (score 80)</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5634,6 +6346,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>support@oncuhome.co.uk</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>https://www.oncuhome.co.uk/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5723,6 +6449,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>info@anteplim.de</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>https://anteplim.de</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5828,6 +6568,20 @@
           <t>Few product links visible; LinkedIn page matched by website</t>
         </is>
       </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>info@freshnuts.de</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>https://freshnuts.de</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5917,6 +6671,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>turkishhome@outlook.de</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>https://turkishhome.de/policies/legal-notice</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6006,6 +6774,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>info@yuvam-moebel.de</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>https://www.cilek-moebel.de</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6091,6 +6873,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>info@istikbal-nrw.de, service@istikbal-nrw.de</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>https://istikbalnrw.com</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6176,6 +6972,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>info@soner.nl</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>https://www.turkse-artikelen.nl</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6269,6 +7079,20 @@
         </is>
       </c>
       <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>info@gultekinbakery.co.uk</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>https://gultekinbakery.co.uk</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6358,6 +7182,12 @@
           <t>LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr"/>
+      <c r="Z64" t="inlineStr"/>
+      <c r="AA64" t="inlineStr"/>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6443,6 +7273,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>info@turkishpantry.co.uk</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>https://turkishpantry.co.uk/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6528,6 +7372,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>info@ozerlat.co.uk, info@ozerlat.com</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>https://ozerlat.co.uk/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr"/>
+      <c r="AB66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6617,6 +7475,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>info@semode.de</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>https://us.semode.de/pages/impressum</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr"/>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6702,6 +7574,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr"/>
+      <c r="Z68" t="inlineStr"/>
+      <c r="AA68" t="inlineStr"/>
+      <c r="AB68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6787,6 +7665,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>support@baklavaciuk.com</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>https://baklavaciuk.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6872,6 +7764,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>deliceland.fr@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>https://deliceland.com/mentions-legales</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6961,6 +7867,20 @@
           <t>LinkedIn page matched by website; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>adm.mediterranee13@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>https://www.istanbul-meuble.fr/contact</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7046,6 +7966,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>info@anteplie.co.uk</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>https://anteplie.co.uk</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7131,6 +8065,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7216,6 +8156,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7305,6 +8251,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>verkauf-ko@best2foryou.de, bellonanrw@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>https://bellonanrw.de</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7394,6 +8354,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>info@serifoglu.nl, shop@serifoglu.nl</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>https://serifoglu.nl/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7479,6 +8453,12 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr"/>
+      <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7564,6 +8544,20 @@
           <t>Turkey-based; EU entity not confirmed; No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>info@b11.com.tr</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>https://www.b11.com.tr</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7649,6 +8643,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>acaciafurnitureuk@gmail.com</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>https://acaciafurniture.uk</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7734,6 +8742,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>info@ihlas.be</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>https://www.ihlas.be/pages/contact</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7823,6 +8845,20 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>info@mobilyum-uk.com</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>https://mobilyum.co.uk</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7912,9 +8948,23 @@
           <t>No verified decision maker found on LinkedIn</t>
         </is>
       </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>info@bellonadeutschland.de</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>https://www.bellonadeutschland.de</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr"/>
+      <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
+      <c r="AC82" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W82"/>
+  <autoFilter ref="A1:AC82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>